<commit_message>
commit realizado em: 2026-10-08
</commit_message>
<xml_diff>
--- a/Metodologias.xlsx
+++ b/Metodologias.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5093564b1391b0aa/Área de Trabalho/POSMARH/Materiais/APP-ÍNDICES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5093564b1391b0aa/Área de Trabalho/POSMARH/Atividades/APP-ÍNDICES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{FC8637FF-0F44-4418-B80D-DD67B6FA12BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3D86F31-7331-4F6B-824F-20519F4A0A7B}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="8_{FC8637FF-0F44-4418-B80D-DD67B6FA12BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{848B81A3-A13B-4349-9595-9F734F858C4D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="135">
   <si>
     <t>Niño 1.2 (°C)</t>
   </si>
@@ -767,6 +767,18 @@
   </si>
   <si>
     <t>The Southwestern South Atlantic (SWSA) mode is characterized by an intense core of SST anomalies extending from the south–southeastern coast of Brazil toward the eastern Atlantic. The SWSA positive phase has a center of positive SST anomalies in the subtropical latitudes and a second one of negative anomalies in the extratropics, whereas the negative phase has the opposite pattern. In Nogueira et al. (2026), it is observed that in South Atlantic Ocean,  except for the first EOF mode (SAD), the remaining EOFs are not independent. Therefore, they applied a Varimax rotation to redistribute the variance and to obtain a monthly pattern more similar to the SWSA mode previously identified by Kayano et al. (2013). It is important to note that the lack of independence becomes irrelevant after applying the rotation.</t>
+  </si>
+  <si>
+    <t>RONI</t>
+  </si>
+  <si>
+    <t>RONI (°C)</t>
+  </si>
+  <si>
+    <t>Relative Oceanic Niño Index</t>
+  </si>
+  <si>
+    <t>The 1991–2020 base period [3 month running mean of ERSST.v5 SST anomalies in the Niño 3.4 region (5°N–5°S, 120°–170°W) with average tropical mean (20°N–20°S) SST anomalies subtracted.</t>
   </si>
 </sst>
 </file>
@@ -1036,10 +1048,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0504FB2E-E332-4BE4-BA95-9AA42EB46B77}" name="Tabela1" displayName="Tabela1" ref="A1:G27" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G27" xr:uid="{0504FB2E-E332-4BE4-BA95-9AA42EB46B77}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G23">
-    <sortCondition ref="A1:A23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0504FB2E-E332-4BE4-BA95-9AA42EB46B77}" name="Tabela1" displayName="Tabela1" ref="A1:G28" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G28" xr:uid="{0504FB2E-E332-4BE4-BA95-9AA42EB46B77}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G24">
+    <sortCondition ref="A1:A24"/>
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3EAE4E6C-889B-48C6-AAF8-DB3BD35DACB1}" name="Index" dataDxfId="6"/>
@@ -1317,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -1476,40 +1488,34 @@
     </row>
     <row r="7" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>7</v>
+        <v>134</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>57</v>
@@ -1524,16 +1530,16 @@
     </row>
     <row r="9" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>57</v>
@@ -1548,16 +1554,16 @@
     </row>
     <row r="10" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>57</v>
@@ -1572,70 +1578,70 @@
     </row>
     <row r="11" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>77</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>92</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>55</v>
@@ -1644,55 +1650,55 @@
     </row>
     <row r="14" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>77</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>125</v>
+        <v>43</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>21</v>
+        <v>125</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>126</v>
+        <v>44</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>127</v>
+        <v>51</v>
       </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>128</v>
+        <v>66</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>77</v>
@@ -1701,10 +1707,10 @@
         <v>21</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>22</v>
@@ -1716,160 +1722,160 @@
     </row>
     <row r="17" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>20</v>
+        <v>127</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>15</v>
@@ -1882,67 +1888,68 @@
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>109</v>
+        <v>13</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>111</v>
+        <v>15</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>112</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>118</v>
+      <c r="C25" s="3" t="s">
+        <v>109</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>114</v>
+        <v>118</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>115</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>6</v>
@@ -1953,19 +1960,19 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>122</v>
+        <v>76</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>114</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>6</v>
@@ -1975,31 +1982,54 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E28" s="6"/>
+      <c r="A28" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E29" s="6"/>
     </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E30" s="6"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F8" r:id="rId1" xr:uid="{AC8C0971-FBAE-4BE0-AAA7-CBC1800B34DC}"/>
-    <hyperlink ref="F9" r:id="rId2" xr:uid="{245EB88A-FE7C-43E9-9638-22C6D9E40350}"/>
-    <hyperlink ref="F10" r:id="rId3" xr:uid="{B9DFECB3-E987-4FF4-9697-4725A45D27B6}"/>
-    <hyperlink ref="F7" r:id="rId4" xr:uid="{ECA62230-534D-4F97-8A6C-63B4E3B96DD4}"/>
-    <hyperlink ref="F20" r:id="rId5" location="SOICALC" display="https://www.cpc.ncep.noaa.gov/data/indices/Readme.index.shtml - SOICALC" xr:uid="{B1D8E77E-2473-482E-BCB2-61498215E874}"/>
-    <hyperlink ref="F23" r:id="rId6" xr:uid="{5C08678B-DCCB-4DB1-A396-05DF1D44A233}"/>
-    <hyperlink ref="F22" r:id="rId7" xr:uid="{414AFD97-2A29-45BD-91E9-7FE87FE43269}"/>
-    <hyperlink ref="F17" r:id="rId8" xr:uid="{7D930AD2-BB31-4516-9F29-81BF351BCDBC}"/>
-    <hyperlink ref="F19" r:id="rId9" xr:uid="{C8785809-3965-4F85-A971-059C01941277}"/>
-    <hyperlink ref="F18" r:id="rId10" xr:uid="{9228F806-3134-4A5D-8563-43A5E0031DB2}"/>
-    <hyperlink ref="F21" r:id="rId11" xr:uid="{A3FDF396-DAE3-42F7-87E6-4CAB4933AD41}"/>
+    <hyperlink ref="F9" r:id="rId1" xr:uid="{AC8C0971-FBAE-4BE0-AAA7-CBC1800B34DC}"/>
+    <hyperlink ref="F10" r:id="rId2" xr:uid="{245EB88A-FE7C-43E9-9638-22C6D9E40350}"/>
+    <hyperlink ref="F11" r:id="rId3" xr:uid="{B9DFECB3-E987-4FF4-9697-4725A45D27B6}"/>
+    <hyperlink ref="F8" r:id="rId4" xr:uid="{ECA62230-534D-4F97-8A6C-63B4E3B96DD4}"/>
+    <hyperlink ref="F21" r:id="rId5" location="SOICALC" display="https://www.cpc.ncep.noaa.gov/data/indices/Readme.index.shtml - SOICALC" xr:uid="{B1D8E77E-2473-482E-BCB2-61498215E874}"/>
+    <hyperlink ref="F24" r:id="rId6" xr:uid="{5C08678B-DCCB-4DB1-A396-05DF1D44A233}"/>
+    <hyperlink ref="F23" r:id="rId7" xr:uid="{414AFD97-2A29-45BD-91E9-7FE87FE43269}"/>
+    <hyperlink ref="F18" r:id="rId8" xr:uid="{7D930AD2-BB31-4516-9F29-81BF351BCDBC}"/>
+    <hyperlink ref="F20" r:id="rId9" xr:uid="{C8785809-3965-4F85-A971-059C01941277}"/>
+    <hyperlink ref="F19" r:id="rId10" xr:uid="{9228F806-3134-4A5D-8563-43A5E0031DB2}"/>
+    <hyperlink ref="F22" r:id="rId11" xr:uid="{A3FDF396-DAE3-42F7-87E6-4CAB4933AD41}"/>
     <hyperlink ref="F5" r:id="rId12" xr:uid="{14120442-89A1-4A75-8BE4-5C765C37105E}"/>
     <hyperlink ref="F4" r:id="rId13" xr:uid="{F20588DE-6804-4152-A357-5A75E889272F}"/>
     <hyperlink ref="F3" r:id="rId14" xr:uid="{0785A3D1-3333-498E-AD13-B78338D847DD}"/>
     <hyperlink ref="F2" r:id="rId15" xr:uid="{1F753BAD-2D85-41DD-8F6B-4B8BF4631DCF}"/>
-    <hyperlink ref="F11" r:id="rId16" xr:uid="{4C36545A-5849-4991-96E7-96B1A53C7F73}"/>
-    <hyperlink ref="F12" r:id="rId17" xr:uid="{46C9D95C-9794-402B-81E1-6EB4A8F03EFD}"/>
-    <hyperlink ref="F13" r:id="rId18" display="https://meteorologia.unifei.edu.br/teleconexoes/indice?id=psa2" xr:uid="{644E1F58-4995-4E43-A95E-032B9E58B994}"/>
+    <hyperlink ref="F12" r:id="rId16" xr:uid="{4C36545A-5849-4991-96E7-96B1A53C7F73}"/>
+    <hyperlink ref="F13" r:id="rId17" xr:uid="{46C9D95C-9794-402B-81E1-6EB4A8F03EFD}"/>
+    <hyperlink ref="F14" r:id="rId18" display="https://meteorologia.unifei.edu.br/teleconexoes/indice?id=psa2" xr:uid="{644E1F58-4995-4E43-A95E-032B9E58B994}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>

</xml_diff>